<commit_message>
samples(lem): the earth dam's five workbooks come from one definition; clay psi is 18, per the source homework
The dam of problems 8 and 16 carried the clay's rapid-drawdown psi as 19 in
three files and 18 in two. The source table (CE 544 rapid drawdown homework)
gives core d = 300 psf, psi = 20 and clay d = 100 psf, psi = 18, shell and sand
blank. The two rapid-drawdown files carry those values; the three steady files
(problem 8 upstream and downstream, problem 16's seepage part) carry none, since
a steady run never reads them. Problem 16's rapid row moves from Bishop 1.120 /
Spencer 1.121 to 1.100 / 1.099 on the same governing circle; every other row is
identical to six decimals. All five files rebuild from benchmarks/build_lem_samples.py;
the seepage sample builders join verify_rebuild.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_gsat_rapid.xlsx
+++ b/docs/lem/files/xslope_gsat_rapid.xlsx
@@ -8572,12 +8572,8 @@
       <c r="I11" s="3">
         <v>0.0</v>
       </c>
-      <c r="J11" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="K11" s="3">
-        <v>0.0</v>
-      </c>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3">
         <v>0.0</v>
@@ -8834,7 +8830,7 @@
         <v>100.0</v>
       </c>
       <c r="K13" s="3">
-        <v>19.0</v>
+        <v>18.0</v>
       </c>
       <c r="L13" s="3"/>
       <c r="M13" s="3">
@@ -8959,12 +8955,8 @@
       <c r="I14" s="3">
         <v>0.0</v>
       </c>
-      <c r="J14" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="K14" s="3">
-        <v>0.0</v>
-      </c>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3">
         <v>0.0</v>

</xml_diff>